<commit_message>
rewired - need QA checks
</commit_message>
<xml_diff>
--- a/data/Access and Willingness to Use (Leb. 2017 - 2021).xlsx
+++ b/data/Access and Willingness to Use (Leb. 2017 - 2021).xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hersheys-my.sharepoint.com/personal/dsmithds_hersheys_com/Documents/misc/lebanon_ctc/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_9676663486020A95DEC6816175FF157340D52A92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56CCAD5B-38FF-4D72-8BDE-8579138585C9}"/>
+  <bookViews>
+    <workbookView xWindow="1320" yWindow="720" windowWidth="15528" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -70,42 +79,48 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -114,7 +129,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -124,62 +139,61 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -369,20 +383,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z64"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="31.5"/>
+    <col min="1" max="1" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -430,24 +447,24 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="8">
-        <v>0.265</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="C2" s="8">
         <v>0.245</v>
       </c>
       <c r="D2" s="8">
-        <v>0.199</v>
+        <v>0.19900000000000001</v>
       </c>
       <c r="E2" s="8">
         <v>0.23</v>
       </c>
       <c r="F2" s="8">
-        <v>0.175</v>
+        <v>0.17499999999999999</v>
       </c>
       <c r="G2" s="8">
         <v>0.156</v>
@@ -459,7 +476,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -470,16 +487,16 @@
         <v>0.158</v>
       </c>
       <c r="D3" s="8">
-        <v>0.119</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="E3" s="8">
         <v>0.152</v>
       </c>
       <c r="F3" s="8">
-        <v>0.118</v>
+        <v>0.11799999999999999</v>
       </c>
       <c r="G3" s="8">
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>11</v>
@@ -488,7 +505,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
@@ -496,19 +513,19 @@
         <v>0.255</v>
       </c>
       <c r="C4" s="8">
-        <v>0.239</v>
+        <v>0.23899999999999999</v>
       </c>
       <c r="D4" s="8">
-        <v>0.206</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="E4" s="8">
-        <v>0.261</v>
+        <v>0.26100000000000001</v>
       </c>
       <c r="F4" s="8">
         <v>0.215</v>
       </c>
       <c r="G4" s="8">
-        <v>0.198</v>
+        <v>0.19800000000000001</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>11</v>
@@ -517,7 +534,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -528,7 +545,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
@@ -536,28 +553,28 @@
         <v>0.499</v>
       </c>
       <c r="C6" s="8">
-        <v>0.469</v>
+        <v>0.46899999999999997</v>
       </c>
       <c r="D6" s="8">
         <v>0.373</v>
       </c>
       <c r="E6" s="8">
-        <v>0.405</v>
+        <v>0.40500000000000003</v>
       </c>
       <c r="F6" s="8">
-        <v>0.365</v>
+        <v>0.36499999999999999</v>
       </c>
       <c r="G6" s="8">
-        <v>0.331</v>
+        <v>0.33100000000000002</v>
       </c>
       <c r="H6" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -571,22 +588,22 @@
         <v>0.247</v>
       </c>
       <c r="E7" s="8">
-        <v>0.265</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="F7" s="8">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="G7" s="8">
-        <v>0.235</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="H7" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>13</v>
       </c>
@@ -594,13 +611,13 @@
         <v>0.38</v>
       </c>
       <c r="C8" s="8">
-        <v>0.343</v>
+        <v>0.34300000000000003</v>
       </c>
       <c r="D8" s="8">
-        <v>0.294</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="E8" s="8">
-        <v>0.328</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="F8" s="8">
         <v>0.308</v>
@@ -609,13 +626,13 @@
         <v>0.317</v>
       </c>
       <c r="H8" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -626,36 +643,36 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="8">
-        <v>0.509</v>
+        <v>0.50900000000000001</v>
       </c>
       <c r="C10" s="8">
         <v>0.5</v>
       </c>
       <c r="D10" s="8">
-        <v>0.414</v>
+        <v>0.41399999999999998</v>
       </c>
       <c r="E10" s="8">
-        <v>0.448</v>
+        <v>0.44800000000000001</v>
       </c>
       <c r="F10" s="8">
-        <v>0.389</v>
+        <v>0.38900000000000001</v>
       </c>
       <c r="G10" s="8">
-        <v>0.336</v>
+        <v>0.33600000000000002</v>
       </c>
       <c r="H10" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -666,54 +683,54 @@
         <v>0.317</v>
       </c>
       <c r="D11" s="8">
-        <v>0.265</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="E11" s="8">
-        <v>0.268</v>
+        <v>0.26800000000000002</v>
       </c>
       <c r="F11" s="8">
-        <v>0.226</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="G11" s="8">
-        <v>0.207</v>
+        <v>0.20699999999999999</v>
       </c>
       <c r="H11" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="8">
-        <v>0.384</v>
+        <v>0.38400000000000001</v>
       </c>
       <c r="C12" s="8">
-        <v>0.346</v>
+        <v>0.34599999999999997</v>
       </c>
       <c r="D12" s="8">
         <v>0.3</v>
       </c>
       <c r="E12" s="8">
-        <v>0.286</v>
+        <v>0.28599999999999998</v>
       </c>
       <c r="F12" s="8">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="G12" s="8">
-        <v>0.306</v>
+        <v>0.30599999999999999</v>
       </c>
       <c r="H12" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -724,36 +741,36 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="8">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="C14" s="8">
         <v>0.438</v>
       </c>
       <c r="D14" s="8">
-        <v>0.347</v>
+        <v>0.34699999999999998</v>
       </c>
       <c r="E14" s="8">
         <v>0.35</v>
       </c>
       <c r="F14" s="8">
-        <v>0.339</v>
+        <v>0.33900000000000002</v>
       </c>
       <c r="G14" s="8">
         <v>0.316</v>
       </c>
       <c r="H14" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>12</v>
       </c>
@@ -764,7 +781,7 @@
         <v>0.317</v>
       </c>
       <c r="D15" s="8">
-        <v>0.237</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="E15" s="8">
         <v>0.253</v>
@@ -773,27 +790,27 @@
         <v>0.253</v>
       </c>
       <c r="G15" s="8">
-        <v>0.237</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="H15" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="8">
-        <v>0.387</v>
+        <v>0.38700000000000001</v>
       </c>
       <c r="C16" s="8">
-        <v>0.339</v>
+        <v>0.33900000000000002</v>
       </c>
       <c r="D16" s="8">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="E16" s="8">
         <v>0.378</v>
@@ -805,13 +822,13 @@
         <v>0.32</v>
       </c>
       <c r="H16" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I16" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -822,7 +839,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>10</v>
       </c>
@@ -845,13 +862,13 @@
         <v>16</v>
       </c>
       <c r="H18" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I18" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>12</v>
       </c>
@@ -874,13 +891,13 @@
         <v>16</v>
       </c>
       <c r="H19" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I19" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>13</v>
       </c>
@@ -903,13 +920,13 @@
         <v>16</v>
       </c>
       <c r="H20" s="9">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="I20" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -920,15 +937,15 @@
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="8">
-        <v>0.349</v>
+        <v>0.34899999999999998</v>
       </c>
       <c r="C22" s="8">
-        <v>0.333</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="D22" s="8">
         <v>0.253</v>
@@ -940,16 +957,16 @@
         <v>0.252</v>
       </c>
       <c r="G22" s="8">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="H22" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>12</v>
       </c>
@@ -960,25 +977,25 @@
         <v>0.222</v>
       </c>
       <c r="D23" s="8">
-        <v>0.149</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="E23" s="8">
         <v>0.219</v>
       </c>
       <c r="F23" s="8">
-        <v>0.176</v>
+        <v>0.17599999999999999</v>
       </c>
       <c r="G23" s="8">
         <v>0.128</v>
       </c>
       <c r="H23" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I23" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>13</v>
       </c>
@@ -986,28 +1003,28 @@
         <v>0.32</v>
       </c>
       <c r="C24" s="8">
-        <v>0.298</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="D24" s="8">
         <v>0.25</v>
       </c>
       <c r="E24" s="8">
-        <v>0.349</v>
+        <v>0.34899999999999998</v>
       </c>
       <c r="F24" s="8">
-        <v>0.295</v>
+        <v>0.29499999999999998</v>
       </c>
       <c r="G24" s="8">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="H24" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I24" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1018,36 +1035,36 @@
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="8">
-        <v>0.364</v>
+        <v>0.36399999999999999</v>
       </c>
       <c r="C26" s="8">
-        <v>0.366</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="D26" s="8">
-        <v>0.275</v>
+        <v>0.27500000000000002</v>
       </c>
       <c r="E26" s="8">
-        <v>0.358</v>
+        <v>0.35799999999999998</v>
       </c>
       <c r="F26" s="8">
-        <v>0.267</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="G26" s="8">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="H26" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I26" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>12</v>
       </c>
@@ -1058,54 +1075,54 @@
         <v>0.223</v>
       </c>
       <c r="D27" s="8">
-        <v>0.163</v>
+        <v>0.16300000000000001</v>
       </c>
       <c r="E27" s="8">
-        <v>0.244</v>
+        <v>0.24399999999999999</v>
       </c>
       <c r="F27" s="8">
-        <v>0.171</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="G27" s="8">
-        <v>0.136</v>
+        <v>0.13600000000000001</v>
       </c>
       <c r="H27" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I27" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B28" s="8">
-        <v>0.338</v>
+        <v>0.33800000000000002</v>
       </c>
       <c r="C28" s="8">
-        <v>0.325</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="D28" s="8">
         <v>0.26</v>
       </c>
       <c r="E28" s="8">
-        <v>0.386</v>
+        <v>0.38600000000000001</v>
       </c>
       <c r="F28" s="8">
-        <v>0.305</v>
+        <v>0.30499999999999999</v>
       </c>
       <c r="G28" s="8">
-        <v>0.235</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="H28" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I28" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -1116,7 +1133,7 @@
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>10</v>
       </c>
@@ -1124,7 +1141,7 @@
         <v>0.31</v>
       </c>
       <c r="C30" s="8">
-        <v>0.301</v>
+        <v>0.30099999999999999</v>
       </c>
       <c r="D30" s="8">
         <v>0.214</v>
@@ -1133,48 +1150,48 @@
         <v>0.251</v>
       </c>
       <c r="F30" s="8">
-        <v>0.234</v>
+        <v>0.23400000000000001</v>
       </c>
       <c r="G30" s="8">
-        <v>0.171</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="H30" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I30" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="8">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="C31" s="8">
         <v>0.22</v>
       </c>
       <c r="D31" s="8">
-        <v>0.134</v>
+        <v>0.13400000000000001</v>
       </c>
       <c r="E31" s="8">
         <v>0.193</v>
       </c>
       <c r="F31" s="8">
-        <v>0.179</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="G31" s="8">
         <v>0.114</v>
       </c>
       <c r="H31" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I31" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>13</v>
       </c>
@@ -1182,28 +1199,28 @@
         <v>0.307</v>
       </c>
       <c r="C32" s="8">
-        <v>0.271</v>
+        <v>0.27100000000000002</v>
       </c>
       <c r="D32" s="8">
-        <v>0.236</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="E32" s="8">
-        <v>0.305</v>
+        <v>0.30499999999999999</v>
       </c>
       <c r="F32" s="8">
-        <v>0.284</v>
+        <v>0.28399999999999997</v>
       </c>
       <c r="G32" s="8">
-        <v>0.233</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="H32" s="9">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I32" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -1214,7 +1231,7 @@
       <c r="H33" s="9"/>
       <c r="I33" s="9"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>10</v>
       </c>
@@ -1228,7 +1245,7 @@
         <v>0.125</v>
       </c>
       <c r="E34" s="8">
-        <v>0.171</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="F34" s="8">
         <v>0.108</v>
@@ -1237,21 +1254,21 @@
         <v>0.112</v>
       </c>
       <c r="H34" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I34" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="8">
-        <v>0.088</v>
+        <v>8.7999999999999995E-2</v>
       </c>
       <c r="C35" s="8">
-        <v>0.074</v>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="D35" s="8">
         <v>0.06</v>
@@ -1260,48 +1277,48 @@
         <v>0.107</v>
       </c>
       <c r="F35" s="8">
-        <v>0.083</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="G35" s="8">
-        <v>0.052</v>
+        <v>5.1999999999999998E-2</v>
       </c>
       <c r="H35" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I35" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B36" s="8">
-        <v>0.203</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="C36" s="8">
-        <v>0.197</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="D36" s="8">
         <v>0.17</v>
       </c>
       <c r="E36" s="8">
-        <v>0.234</v>
+        <v>0.23400000000000001</v>
       </c>
       <c r="F36" s="8">
         <v>0.184</v>
       </c>
       <c r="G36" s="8">
-        <v>0.169</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="H36" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I36" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="7"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -1312,70 +1329,70 @@
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B38" s="8">
-        <v>0.166</v>
+        <v>0.16600000000000001</v>
       </c>
       <c r="C38" s="8">
-        <v>0.137</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="D38" s="8">
-        <v>0.139</v>
+        <v>0.13900000000000001</v>
       </c>
       <c r="E38" s="8">
         <v>0.186</v>
       </c>
       <c r="F38" s="8">
-        <v>0.144</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="G38" s="8">
         <v>0.12</v>
       </c>
       <c r="H38" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I38" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="8">
-        <v>0.083</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="C39" s="8">
-        <v>0.076</v>
+        <v>7.5999999999999998E-2</v>
       </c>
       <c r="D39" s="8">
-        <v>0.067</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="E39" s="8">
         <v>0.115</v>
       </c>
       <c r="F39" s="8">
-        <v>0.089</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="G39" s="8">
-        <v>0.059</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="H39" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I39" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B40" s="8">
-        <v>0.226</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="C40" s="8">
         <v>0.215</v>
@@ -1390,16 +1407,16 @@
         <v>0.217</v>
       </c>
       <c r="G40" s="8">
-        <v>0.144</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="H40" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I40" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -1410,7 +1427,7 @@
       <c r="H41" s="9"/>
       <c r="I41" s="9"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>10</v>
       </c>
@@ -1427,19 +1444,19 @@
         <v>0.156</v>
       </c>
       <c r="F42" s="8">
-        <v>0.069</v>
+        <v>6.9000000000000006E-2</v>
       </c>
       <c r="G42" s="8">
-        <v>0.096</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H42" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I42" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>12</v>
       </c>
@@ -1447,36 +1464,36 @@
         <v>0.08</v>
       </c>
       <c r="C43" s="8">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D43" s="8">
-        <v>0.046</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="E43" s="8">
-        <v>0.103</v>
+        <v>0.10299999999999999</v>
       </c>
       <c r="F43" s="8">
-        <v>0.074</v>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="G43" s="8">
-        <v>0.038</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="H43" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I43" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B44" s="8">
-        <v>0.194</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="C44" s="8">
-        <v>0.179</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="D44" s="8">
         <v>0.153</v>
@@ -1488,16 +1505,16 @@
         <v>0.153</v>
       </c>
       <c r="G44" s="8">
-        <v>0.174</v>
+        <v>0.17399999999999999</v>
       </c>
       <c r="H44" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I44" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="7"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -1508,7 +1525,7 @@
       <c r="H45" s="9"/>
       <c r="I45" s="9"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
         <v>10</v>
       </c>
@@ -1519,7 +1536,7 @@
         <v>16</v>
       </c>
       <c r="D46" s="8">
-        <v>0.209</v>
+        <v>0.20899999999999999</v>
       </c>
       <c r="E46" s="9" t="s">
         <v>16</v>
@@ -1528,16 +1545,16 @@
         <v>16</v>
       </c>
       <c r="G46" s="8">
-        <v>0.293</v>
+        <v>0.29299999999999998</v>
       </c>
       <c r="H46" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I46" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>12</v>
       </c>
@@ -1548,7 +1565,7 @@
         <v>16</v>
       </c>
       <c r="D47" s="8">
-        <v>0.144</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>16</v>
@@ -1557,16 +1574,16 @@
         <v>16</v>
       </c>
       <c r="G47" s="8">
-        <v>0.195</v>
+        <v>0.19500000000000001</v>
       </c>
       <c r="H47" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I47" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>13</v>
       </c>
@@ -1577,7 +1594,7 @@
         <v>16</v>
       </c>
       <c r="D48" s="8">
-        <v>0.298</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="E48" s="9" t="s">
         <v>16</v>
@@ -1586,16 +1603,16 @@
         <v>16</v>
       </c>
       <c r="G48" s="8">
-        <v>0.425</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="H48" s="9">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="I48" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="7"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -1606,94 +1623,94 @@
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B50" s="8">
-        <v>0.042</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="C50" s="8">
-        <v>0.045</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="D50" s="8">
-        <v>0.042</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="E50" s="8">
-        <v>0.041</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="F50" s="8">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="G50" s="8">
-        <v>0.039</v>
+        <v>3.9E-2</v>
       </c>
       <c r="H50" s="9">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I50" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B51" s="8">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="C51" s="8">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="D51" s="8">
-        <v>0.014</v>
+        <v>1.4E-2</v>
       </c>
       <c r="E51" s="8">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F51" s="8">
-        <v>0.011</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="G51" s="8">
-        <v>0.008</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="H51" s="9">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I51" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B52" s="8">
-        <v>0.082</v>
+        <v>8.2000000000000003E-2</v>
       </c>
       <c r="C52" s="8">
-        <v>0.101</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="D52" s="8">
         <v>0.09</v>
       </c>
       <c r="E52" s="8">
-        <v>0.073</v>
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="F52" s="8">
-        <v>0.088</v>
+        <v>8.7999999999999995E-2</v>
       </c>
       <c r="G52" s="8">
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="H52" s="9">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I52" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="7"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -1704,27 +1721,27 @@
       <c r="H53" s="9"/>
       <c r="I53" s="9"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B54" s="8">
-        <v>0.261</v>
+        <v>0.26100000000000001</v>
       </c>
       <c r="C54" s="8">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="D54" s="8">
-        <v>0.208</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="E54" s="8">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="F54" s="8">
-        <v>0.194</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="G54" s="8">
-        <v>0.165</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>11</v>
@@ -1733,7 +1750,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>12</v>
       </c>
@@ -1747,13 +1764,13 @@
         <v>0.12</v>
       </c>
       <c r="E55" s="8">
-        <v>0.167</v>
+        <v>0.16700000000000001</v>
       </c>
       <c r="F55" s="8">
-        <v>0.116</v>
+        <v>0.11600000000000001</v>
       </c>
       <c r="G55" s="8">
-        <v>0.093</v>
+        <v>9.2999999999999999E-2</v>
       </c>
       <c r="H55" s="9" t="s">
         <v>11</v>
@@ -1762,18 +1779,18 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B56" s="8">
-        <v>0.264</v>
+        <v>0.26400000000000001</v>
       </c>
       <c r="C56" s="8">
         <v>0.251</v>
       </c>
       <c r="D56" s="8">
-        <v>0.208</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="E56" s="8">
         <v>0.27</v>
@@ -1791,7 +1808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
@@ -1802,27 +1819,27 @@
       <c r="H57" s="9"/>
       <c r="I57" s="9"/>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="11">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="C58" s="11">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="D58" s="11">
-        <v>0.168</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="E58" s="11">
-        <v>0.196</v>
+        <v>0.19600000000000001</v>
       </c>
       <c r="F58" s="11">
         <v>0.155</v>
       </c>
       <c r="G58" s="11">
-        <v>0.138</v>
+        <v>0.13800000000000001</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>11</v>
@@ -1831,27 +1848,27 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B59" s="11">
-        <v>0.149</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="C59" s="11">
         <v>0.157</v>
       </c>
       <c r="D59" s="11">
-        <v>0.099</v>
+        <v>9.9000000000000005E-2</v>
       </c>
       <c r="E59" s="11">
-        <v>0.137</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="F59" s="11">
-        <v>0.119</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="G59" s="11">
-        <v>0.086</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="H59" s="9" t="s">
         <v>11</v>
@@ -1860,7 +1877,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>13</v>
       </c>
@@ -1868,7 +1885,7 @@
         <v>0.246</v>
       </c>
       <c r="C60" s="11">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="D60" s="11">
         <v>0.187</v>
@@ -1877,10 +1894,10 @@
         <v>0.252</v>
       </c>
       <c r="F60" s="11">
-        <v>0.208</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="G60" s="11">
-        <v>0.196</v>
+        <v>0.19600000000000001</v>
       </c>
       <c r="H60" s="9" t="s">
         <v>11</v>
@@ -1889,7 +1906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A61" s="7"/>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
@@ -1900,7 +1917,7 @@
       <c r="H61" s="9"/>
       <c r="I61" s="9"/>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A62" s="7" t="s">
         <v>10</v>
       </c>
@@ -1911,7 +1928,7 @@
         <v>16</v>
       </c>
       <c r="D62" s="8">
-        <v>0.243</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>16</v>
@@ -1920,7 +1937,7 @@
         <v>16</v>
       </c>
       <c r="G62" s="8">
-        <v>0.293</v>
+        <v>0.29299999999999998</v>
       </c>
       <c r="H62" s="9" t="s">
         <v>11</v>
@@ -1929,7 +1946,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>12</v>
       </c>
@@ -1949,7 +1966,7 @@
         <v>16</v>
       </c>
       <c r="G63" s="8">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>11</v>
@@ -1958,7 +1975,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>13</v>
       </c>
@@ -1978,7 +1995,7 @@
         <v>16</v>
       </c>
       <c r="G64" s="8">
-        <v>0.346</v>
+        <v>0.34599999999999997</v>
       </c>
       <c r="H64" s="9" t="s">
         <v>11</v>
@@ -1988,6 +2005,12 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{ecb9909e-a632-4cc5-be2e-ce284d9ed345}" enabled="1" method="Standard" siteId="{90254b37-ddd6-4784-a73c-67a28484e423}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>